<commit_message>
Aplica identidade visual Meliuz ao painel
</commit_message>
<xml_diff>
--- a/saidas/painel_meliuz.xlsx
+++ b/saidas/painel_meliuz.xlsx
@@ -22,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="R$ #,##0.00"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,7 +37,12 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="0017365D"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0031583A"/>
       <sz val="13"/>
     </font>
     <font>
@@ -45,14 +50,14 @@
       <color rgb="00FFFFFF"/>
     </font>
     <font>
-      <color rgb="0044546A"/>
+      <color rgb="0034423A"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="0017365D"/>
+      <color rgb="0031583A"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -61,32 +66,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F6F8FB"/>
+        <fgColor rgb="00F5F7F5"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0017365D"/>
+        <fgColor rgb="00426F49"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DDEBF7"/>
+        <fgColor rgb="00FCE4EF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2F0D9"/>
+        <fgColor rgb="00E7F1E7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00548235"/>
+        <fgColor rgb="00FFF0C7"/>
       </patternFill>
     </fill>
     <fill>
@@ -119,16 +119,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D9E2F3"/>
+        <color rgb="00D8E3D8"/>
       </left>
       <right style="thin">
-        <color rgb="00D9E2F3"/>
+        <color rgb="00D8E3D8"/>
       </right>
       <top style="thin">
-        <color rgb="00D9E2F3"/>
+        <color rgb="00D8E3D8"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9E2F3"/>
+        <color rgb="00D8E3D8"/>
       </bottom>
     </border>
   </borders>
@@ -137,51 +137,51 @@
   </cellStyleXfs>
   <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="4" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="5" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -266,10 +266,10 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>13</row>
+      <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5334000" cy="2857500"/>
+    <ext cx="400050" cy="400050"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -289,12 +289,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>6</col>
+      <col>0</col>
       <colOff>0</colOff>
-      <row>13</row>
+      <row>14</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5334000" cy="2857500"/>
+    <ext cx="5429250" cy="2905125"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -312,6 +312,31 @@
     </pic>
     <clientData/>
   </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5429250" cy="2905125"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -319,12 +344,12 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>9</col>
+      <col>0</col>
       <colOff>0</colOff>
-      <row>2</row>
+      <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4953000" cy="2714625"/>
+    <ext cx="400050" cy="400050"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -346,7 +371,7 @@
     <from>
       <col>9</col>
       <colOff>0</colOff>
-      <row>18</row>
+      <row>3</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="4953000" cy="2714625"/>
@@ -367,6 +392,31 @@
     </pic>
     <clientData/>
   </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4953000" cy="2714625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -374,12 +424,12 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>9</col>
+      <col>0</col>
       <colOff>0</colOff>
-      <row>2</row>
+      <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4953000" cy="2714625"/>
+    <ext cx="400050" cy="400050"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -401,7 +451,7 @@
     <from>
       <col>9</col>
       <colOff>0</colOff>
-      <row>18</row>
+      <row>3</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="4953000" cy="2714625"/>
@@ -422,6 +472,31 @@
     </pic>
     <clientData/>
   </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4953000" cy="2714625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -429,12 +504,12 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>9</col>
+      <col>0</col>
       <colOff>0</colOff>
-      <row>2</row>
+      <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4953000" cy="2714625"/>
+    <ext cx="400050" cy="400050"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -456,7 +531,7 @@
     <from>
       <col>9</col>
       <colOff>0</colOff>
-      <row>18</row>
+      <row>3</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="4953000" cy="2714625"/>
@@ -467,6 +542,31 @@
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4953000" cy="2714625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -800,10 +900,11 @@
     <col width="12" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Dashboard de Testes A/B de Cashback</t>
+          <t xml:space="preserve">     Dashboard de Testes A/B de Cashback
+     Analise automatizada de testes de cashback</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -832,19 +933,19 @@
       <c r="Y1" s="3" t="n"/>
       <c r="Z1" s="3" t="n"/>
     </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="3" t="n"/>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="3" t="n"/>
-      <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="n"/>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
       <c r="M2" s="3" t="n"/>
       <c r="N2" s="3" t="n"/>
       <c r="O2" s="3" t="n"/>
@@ -860,39 +961,19 @@
       <c r="Y2" s="3" t="n"/>
       <c r="Z2" s="3" t="n"/>
     </row>
-    <row r="3" ht="27" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Testes analisados
-3</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="n"/>
-      <c r="C3" s="5" t="n"/>
-      <c r="D3" s="6" t="inlineStr">
-        <is>
-          <t>Lucro vencedor total
-R$ 726.050,00</t>
-        </is>
-      </c>
-      <c r="E3" s="7" t="n"/>
-      <c r="F3" s="7" t="n"/>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>Margem media
-5,41%</t>
-        </is>
-      </c>
-      <c r="H3" s="9" t="n"/>
-      <c r="I3" s="9" t="n"/>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>ROI medio
-129,46%</t>
-        </is>
-      </c>
-      <c r="K3" s="5" t="n"/>
-      <c r="L3" s="5" t="n"/>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="3" t="n"/>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="3" t="n"/>
+      <c r="F3" s="3" t="n"/>
+      <c r="G3" s="3" t="n"/>
+      <c r="H3" s="3" t="n"/>
+      <c r="I3" s="3" t="n"/>
+      <c r="J3" s="3" t="n"/>
+      <c r="K3" s="3" t="n"/>
+      <c r="L3" s="3" t="n"/>
       <c r="M3" s="3" t="n"/>
       <c r="N3" s="3" t="n"/>
       <c r="O3" s="3" t="n"/>
@@ -909,16 +990,36 @@
       <c r="Z3" s="3" t="n"/>
     </row>
     <row r="4" ht="27" customHeight="1">
-      <c r="A4" s="5" t="n"/>
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Testes analisados
+3</t>
+        </is>
+      </c>
       <c r="B4" s="5" t="n"/>
       <c r="C4" s="5" t="n"/>
-      <c r="D4" s="7" t="n"/>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Lucro vencedor total
+R$ 726.050,00</t>
+        </is>
+      </c>
       <c r="E4" s="7" t="n"/>
       <c r="F4" s="7" t="n"/>
-      <c r="G4" s="9" t="n"/>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>Margem media
+5,41%</t>
+        </is>
+      </c>
       <c r="H4" s="9" t="n"/>
       <c r="I4" s="9" t="n"/>
-      <c r="J4" s="5" t="n"/>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>ROI medio
+129,46%</t>
+        </is>
+      </c>
       <c r="K4" s="5" t="n"/>
       <c r="L4" s="5" t="n"/>
       <c r="M4" s="3" t="n"/>
@@ -964,19 +1065,19 @@
       <c r="Y5" s="3" t="n"/>
       <c r="Z5" s="3" t="n"/>
     </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="3" t="n"/>
-      <c r="B6" s="3" t="n"/>
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
-      <c r="F6" s="3" t="n"/>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
-      <c r="I6" s="3" t="n"/>
-      <c r="J6" s="3" t="n"/>
-      <c r="K6" s="3" t="n"/>
-      <c r="L6" s="3" t="n"/>
+    <row r="6" ht="27" customHeight="1">
+      <c r="A6" s="5" t="n"/>
+      <c r="B6" s="5" t="n"/>
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="7" t="n"/>
+      <c r="E6" s="7" t="n"/>
+      <c r="F6" s="7" t="n"/>
+      <c r="G6" s="9" t="n"/>
+      <c r="H6" s="9" t="n"/>
+      <c r="I6" s="9" t="n"/>
+      <c r="J6" s="5" t="n"/>
+      <c r="K6" s="5" t="n"/>
+      <c r="L6" s="5" t="n"/>
       <c r="M6" s="3" t="n"/>
       <c r="N6" s="3" t="n"/>
       <c r="O6" s="3" t="n"/>
@@ -1021,41 +1122,13 @@
       <c r="Z7" s="3" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>Parceiro</t>
-        </is>
-      </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>Periodo</t>
-        </is>
-      </c>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>Variante</t>
-        </is>
-      </c>
-      <c r="D8" s="10" t="inlineStr">
-        <is>
-          <t>Lucro</t>
-        </is>
-      </c>
-      <c r="E8" s="10" t="inlineStr">
-        <is>
-          <t>Margem</t>
-        </is>
-      </c>
-      <c r="F8" s="10" t="inlineStr">
-        <is>
-          <t>ROI</t>
-        </is>
-      </c>
-      <c r="G8" s="10" t="inlineStr">
-        <is>
-          <t>Decisao</t>
-        </is>
-      </c>
+      <c r="A8" s="3" t="n"/>
+      <c r="B8" s="3" t="n"/>
+      <c r="C8" s="3" t="n"/>
+      <c r="D8" s="3" t="n"/>
+      <c r="E8" s="3" t="n"/>
+      <c r="F8" s="3" t="n"/>
+      <c r="G8" s="3" t="n"/>
       <c r="H8" s="3" t="n"/>
       <c r="I8" s="3" t="n"/>
       <c r="J8" s="3" t="n"/>
@@ -1076,34 +1149,40 @@
       <c r="Y8" s="3" t="n"/>
       <c r="Z8" s="3" t="n"/>
     </row>
-    <row r="9" ht="38" customHeight="1">
-      <c r="A9" s="11" t="inlineStr">
-        <is>
-          <t>Parceiro A</t>
-        </is>
-      </c>
-      <c r="B9" s="11" t="inlineStr">
-        <is>
-          <t>2011-01-01 a 2011-04-02</t>
-        </is>
-      </c>
-      <c r="C9" s="11" t="inlineStr">
-        <is>
-          <t>Grupo 1</t>
-        </is>
-      </c>
-      <c r="D9" s="12" t="n">
-        <v>404711</v>
-      </c>
-      <c r="E9" s="13" t="n">
-        <v>0.07220312379296767</v>
-      </c>
-      <c r="F9" s="13" t="n">
-        <v>1.733802008362465</v>
-      </c>
-      <c r="G9" s="11" t="inlineStr">
-        <is>
-          <t>Escalar Grupo 1 para 100% do trafego, mantendo monitoramento de margem e cashback pago nos primeiros dias.</t>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Parceiro</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Periodo</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Variante</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>Lucro</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>Margem</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>ROI</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>Decisao</t>
         </is>
       </c>
       <c r="H9" s="3" t="n"/>
@@ -1129,12 +1208,12 @@
     <row r="10" ht="38" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>Parceiro B</t>
+          <t>Parceiro A</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>2011-05-01 a 2011-06-30</t>
+          <t>2011-01-01 a 2011-04-02</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
@@ -1143,13 +1222,13 @@
         </is>
       </c>
       <c r="D10" s="12" t="n">
-        <v>286570</v>
+        <v>404711</v>
       </c>
       <c r="E10" s="13" t="n">
-        <v>0.07000066930185954</v>
+        <v>0.07220312379296767</v>
       </c>
       <c r="F10" s="13" t="n">
-        <v>1.750035114289378</v>
+        <v>1.733802008362465</v>
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
@@ -1179,12 +1258,12 @@
     <row r="11" ht="38" customHeight="1">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>Parceiro C</t>
+          <t>Parceiro B</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>2011-07-01 a 2011-08-14</t>
+          <t>2011-05-01 a 2011-06-30</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
@@ -1193,13 +1272,13 @@
         </is>
       </c>
       <c r="D11" s="12" t="n">
-        <v>34769</v>
+        <v>286570</v>
       </c>
       <c r="E11" s="13" t="n">
-        <v>0.0199998849556504</v>
+        <v>0.07000066930185954</v>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.3999930974184345</v>
+        <v>1.750035114289378</v>
       </c>
       <c r="G11" s="11" t="inlineStr">
         <is>
@@ -1226,14 +1305,36 @@
       <c r="Y11" s="3" t="n"/>
       <c r="Z11" s="3" t="n"/>
     </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="3" t="n"/>
-      <c r="B12" s="3" t="n"/>
-      <c r="C12" s="3" t="n"/>
-      <c r="D12" s="3" t="n"/>
-      <c r="E12" s="3" t="n"/>
-      <c r="F12" s="3" t="n"/>
-      <c r="G12" s="3" t="n"/>
+    <row r="12" ht="38" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>Parceiro C</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>2011-07-01 a 2011-08-14</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Grupo 1</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="n">
+        <v>34769</v>
+      </c>
+      <c r="E12" s="13" t="n">
+        <v>0.0199998849556504</v>
+      </c>
+      <c r="F12" s="13" t="n">
+        <v>0.3999930974184345</v>
+      </c>
+      <c r="G12" s="11" t="inlineStr">
+        <is>
+          <t>Escalar Grupo 1 para 100% do trafego, mantendo monitoramento de margem e cashback pago nos primeiros dias.</t>
+        </is>
+      </c>
       <c r="H12" s="3" t="n"/>
       <c r="I12" s="3" t="n"/>
       <c r="J12" s="3" t="n"/>
@@ -4280,11 +4381,11 @@
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="D3:F5"/>
-    <mergeCell ref="J3:L5"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="G3:I5"/>
-    <mergeCell ref="A3:C5"/>
+    <mergeCell ref="G4:I6"/>
+    <mergeCell ref="J4:L6"/>
+    <mergeCell ref="A1:L2"/>
+    <mergeCell ref="A4:C6"/>
+    <mergeCell ref="D4:F6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4328,10 +4429,11 @@
     <col width="12" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Teste cashback - Parceiro A</t>
+          <t xml:space="preserve">     Teste cashback - Parceiro A
+     2011-01-01 a 2011-04-02 | decisao automatizada</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -4364,21 +4466,21 @@
       <c r="Y1" s="3" t="n"/>
       <c r="Z1" s="3" t="n"/>
     </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="3" t="n"/>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="3" t="n"/>
-      <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="n"/>
-      <c r="M2" s="3" t="n"/>
-      <c r="N2" s="3" t="n"/>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
       <c r="O2" s="3" t="n"/>
       <c r="P2" s="3" t="n"/>
       <c r="Q2" s="3" t="n"/>
@@ -4392,35 +4494,15 @@
       <c r="Y2" s="3" t="n"/>
       <c r="Z2" s="3" t="n"/>
     </row>
-    <row r="3" ht="27" customHeight="1">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>Variante recomendada
-Grupo 1</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="n"/>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>Lucro liquido
-R$ 404.711,00</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="n"/>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>Margem GMV
-7,22%</t>
-        </is>
-      </c>
-      <c r="F3" s="9" t="n"/>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>ROI cashback
-173,38%</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="n"/>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="3" t="n"/>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="3" t="n"/>
+      <c r="F3" s="3" t="n"/>
+      <c r="G3" s="3" t="n"/>
+      <c r="H3" s="3" t="n"/>
       <c r="I3" s="3" t="n"/>
       <c r="J3" s="3" t="n"/>
       <c r="K3" s="3" t="n"/>
@@ -4457,13 +4539,33 @@
       <c r="Z3" s="3" t="n"/>
     </row>
     <row r="4" ht="27" customHeight="1">
-      <c r="A4" s="7" t="n"/>
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Variante recomendada
+Grupo 1</t>
+        </is>
+      </c>
       <c r="B4" s="7" t="n"/>
-      <c r="C4" s="7" t="n"/>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Lucro liquido
+R$ 404.711,00</t>
+        </is>
+      </c>
       <c r="D4" s="7" t="n"/>
-      <c r="E4" s="9" t="n"/>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Margem GMV
+7,22%</t>
+        </is>
+      </c>
       <c r="F4" s="9" t="n"/>
-      <c r="G4" s="5" t="n"/>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>ROI cashback
+173,38%</t>
+        </is>
+      </c>
       <c r="H4" s="5" t="n"/>
       <c r="I4" s="3" t="n"/>
       <c r="J4" s="3" t="n"/>
@@ -4532,15 +4634,15 @@
       <c r="Y5" s="3" t="n"/>
       <c r="Z5" s="3" t="n"/>
     </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="3" t="n"/>
-      <c r="B6" s="3" t="n"/>
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
-      <c r="F6" s="3" t="n"/>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
+    <row r="6" ht="27" customHeight="1">
+      <c r="A6" s="7" t="n"/>
+      <c r="B6" s="7" t="n"/>
+      <c r="C6" s="7" t="n"/>
+      <c r="D6" s="7" t="n"/>
+      <c r="E6" s="9" t="n"/>
+      <c r="F6" s="9" t="n"/>
+      <c r="G6" s="5" t="n"/>
+      <c r="H6" s="5" t="n"/>
       <c r="I6" s="3" t="n"/>
       <c r="J6" s="3" t="n"/>
       <c r="K6" s="3" t="n"/>
@@ -4571,22 +4673,14 @@
       <c r="Z6" s="3" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="16" t="inlineStr">
-        <is>
-          <t>Decisao</t>
-        </is>
-      </c>
-      <c r="B7" s="17" t="inlineStr">
-        <is>
-          <t>Escalar Grupo 1 para 100% do trafego, mantendo monitoramento de margem e cashback pago nos primeiros dias.</t>
-        </is>
-      </c>
-      <c r="C7" s="18" t="n"/>
-      <c r="D7" s="18" t="n"/>
-      <c r="E7" s="18" t="n"/>
-      <c r="F7" s="18" t="n"/>
-      <c r="G7" s="18" t="n"/>
-      <c r="H7" s="18" t="n"/>
+      <c r="A7" s="3" t="n"/>
+      <c r="B7" s="3" t="n"/>
+      <c r="C7" s="3" t="n"/>
+      <c r="D7" s="3" t="n"/>
+      <c r="E7" s="3" t="n"/>
+      <c r="F7" s="3" t="n"/>
+      <c r="G7" s="3" t="n"/>
+      <c r="H7" s="3" t="n"/>
       <c r="I7" s="3" t="n"/>
       <c r="J7" s="3" t="n"/>
       <c r="K7" s="3" t="n"/>
@@ -4617,8 +4711,16 @@
       <c r="Z7" s="3" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="18" t="n"/>
-      <c r="B8" s="18" t="n"/>
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>Decisao</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>Escalar Grupo 1 para 100% do trafego, mantendo monitoramento de margem e cashback pago nos primeiros dias.</t>
+        </is>
+      </c>
       <c r="C8" s="18" t="n"/>
       <c r="D8" s="18" t="n"/>
       <c r="E8" s="18" t="n"/>
@@ -4655,14 +4757,14 @@
       <c r="Z8" s="3" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="3" t="n"/>
-      <c r="B9" s="3" t="n"/>
-      <c r="C9" s="3" t="n"/>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
-      <c r="F9" s="3" t="n"/>
-      <c r="G9" s="3" t="n"/>
-      <c r="H9" s="3" t="n"/>
+      <c r="A9" s="18" t="n"/>
+      <c r="B9" s="18" t="n"/>
+      <c r="C9" s="18" t="n"/>
+      <c r="D9" s="18" t="n"/>
+      <c r="E9" s="18" t="n"/>
+      <c r="F9" s="18" t="n"/>
+      <c r="G9" s="18" t="n"/>
+      <c r="H9" s="18" t="n"/>
       <c r="I9" s="3" t="n"/>
       <c r="J9" s="3" t="n"/>
       <c r="K9" s="3" t="n"/>
@@ -4731,46 +4833,14 @@
       <c r="Z10" s="3" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>Grupo</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>Compradores</t>
-        </is>
-      </c>
-      <c r="C11" s="10" t="inlineStr">
-        <is>
-          <t>GMV</t>
-        </is>
-      </c>
-      <c r="D11" s="10" t="inlineStr">
-        <is>
-          <t>Cashback</t>
-        </is>
-      </c>
-      <c r="E11" s="10" t="inlineStr">
-        <is>
-          <t>Lucro</t>
-        </is>
-      </c>
-      <c r="F11" s="10" t="inlineStr">
-        <is>
-          <t>Margem</t>
-        </is>
-      </c>
-      <c r="G11" s="10" t="inlineStr">
-        <is>
-          <t>ROI</t>
-        </is>
-      </c>
-      <c r="H11" s="10" t="inlineStr">
-        <is>
-          <t>Ticket medio</t>
-        </is>
-      </c>
+      <c r="A11" s="3" t="n"/>
+      <c r="B11" s="3" t="n"/>
+      <c r="C11" s="3" t="n"/>
+      <c r="D11" s="3" t="n"/>
+      <c r="E11" s="3" t="n"/>
+      <c r="F11" s="3" t="n"/>
+      <c r="G11" s="3" t="n"/>
+      <c r="H11" s="3" t="n"/>
       <c r="I11" s="3" t="n"/>
       <c r="J11" s="3" t="n"/>
       <c r="K11" s="3" t="n"/>
@@ -4801,31 +4871,45 @@
       <c r="Z11" s="3" t="n"/>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>Grupo 1</t>
-        </is>
-      </c>
-      <c r="B12" s="19" t="n">
-        <v>9633</v>
-      </c>
-      <c r="C12" s="20" t="n">
-        <v>5605173</v>
-      </c>
-      <c r="D12" s="20" t="n">
-        <v>233424</v>
-      </c>
-      <c r="E12" s="20" t="n">
-        <v>404711</v>
-      </c>
-      <c r="F12" s="21" t="n">
-        <v>0.07220312379296767</v>
-      </c>
-      <c r="G12" s="21" t="n">
-        <v>1.733802008362465</v>
-      </c>
-      <c r="H12" s="20" t="n">
-        <v>581.8720024914356</v>
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Grupo</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Compradores</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>GMV</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>Cashback</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>Lucro</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>Margem</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>ROI</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>Ticket medio</t>
+        </is>
       </c>
       <c r="I12" s="3" t="n"/>
       <c r="J12" s="3" t="n"/>
@@ -4857,31 +4941,31 @@
       <c r="Z12" s="3" t="n"/>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="11" t="inlineStr">
-        <is>
-          <t>Grupo 2</t>
-        </is>
-      </c>
-      <c r="B13" s="11" t="n">
-        <v>10814</v>
-      </c>
-      <c r="C13" s="12" t="n">
-        <v>6423096</v>
-      </c>
-      <c r="D13" s="12" t="n">
-        <v>370659</v>
-      </c>
-      <c r="E13" s="12" t="n">
-        <v>357519</v>
-      </c>
-      <c r="F13" s="13" t="n">
-        <v>0.05566147540064791</v>
-      </c>
-      <c r="G13" s="13" t="n">
-        <v>0.9645496264760872</v>
-      </c>
-      <c r="H13" s="12" t="n">
-        <v>593.9611614573701</v>
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>Grupo 1</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="n">
+        <v>9633</v>
+      </c>
+      <c r="C13" s="20" t="n">
+        <v>5605173</v>
+      </c>
+      <c r="D13" s="20" t="n">
+        <v>233424</v>
+      </c>
+      <c r="E13" s="20" t="n">
+        <v>404711</v>
+      </c>
+      <c r="F13" s="21" t="n">
+        <v>0.07220312379296767</v>
+      </c>
+      <c r="G13" s="21" t="n">
+        <v>1.733802008362465</v>
+      </c>
+      <c r="H13" s="20" t="n">
+        <v>581.8720024914356</v>
       </c>
       <c r="I13" s="3" t="n"/>
       <c r="J13" s="3" t="n"/>
@@ -4915,29 +4999,29 @@
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>Grupo 3</t>
+          <t>Grupo 2</t>
         </is>
       </c>
       <c r="B14" s="11" t="n">
-        <v>11410</v>
+        <v>10814</v>
       </c>
       <c r="C14" s="12" t="n">
-        <v>6785856</v>
+        <v>6423096</v>
       </c>
       <c r="D14" s="12" t="n">
-        <v>503600</v>
+        <v>370659</v>
       </c>
       <c r="E14" s="12" t="n">
-        <v>264287</v>
+        <v>357519</v>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.03894674452272492</v>
+        <v>0.05566147540064791</v>
       </c>
       <c r="G14" s="13" t="n">
-        <v>0.5247954725972994</v>
+        <v>0.9645496264760872</v>
       </c>
       <c r="H14" s="12" t="n">
-        <v>594.7288343558282</v>
+        <v>593.9611614573701</v>
       </c>
       <c r="I14" s="3" t="n"/>
       <c r="J14" s="3" t="n"/>
@@ -4969,14 +5053,32 @@
       <c r="Z14" s="3" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="3" t="n"/>
-      <c r="B15" s="3" t="n"/>
-      <c r="C15" s="3" t="n"/>
-      <c r="D15" s="3" t="n"/>
-      <c r="E15" s="3" t="n"/>
-      <c r="F15" s="3" t="n"/>
-      <c r="G15" s="3" t="n"/>
-      <c r="H15" s="3" t="n"/>
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>Grupo 3</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="n">
+        <v>11410</v>
+      </c>
+      <c r="C15" s="12" t="n">
+        <v>6785856</v>
+      </c>
+      <c r="D15" s="12" t="n">
+        <v>503600</v>
+      </c>
+      <c r="E15" s="12" t="n">
+        <v>264287</v>
+      </c>
+      <c r="F15" s="13" t="n">
+        <v>0.03894674452272492</v>
+      </c>
+      <c r="G15" s="13" t="n">
+        <v>0.5247954725972994</v>
+      </c>
+      <c r="H15" s="12" t="n">
+        <v>594.7288343558282</v>
+      </c>
       <c r="I15" s="3" t="n"/>
       <c r="J15" s="3" t="n"/>
       <c r="K15" s="3" t="n"/>
@@ -8748,12 +8850,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A1:N1"/>
-    <mergeCell ref="A3:B5"/>
-    <mergeCell ref="G3:H5"/>
-    <mergeCell ref="E3:F5"/>
-    <mergeCell ref="B7:H8"/>
-    <mergeCell ref="C3:D5"/>
+    <mergeCell ref="A1:N2"/>
+    <mergeCell ref="E4:F6"/>
+    <mergeCell ref="B8:H9"/>
+    <mergeCell ref="C4:D6"/>
+    <mergeCell ref="A4:B6"/>
+    <mergeCell ref="G4:H6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -8797,10 +8899,11 @@
     <col width="12" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Teste cashback - Parceiro B</t>
+          <t xml:space="preserve">     Teste cashback - Parceiro B
+     2011-05-01 a 2011-06-30 | decisao automatizada</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -8833,21 +8936,21 @@
       <c r="Y1" s="3" t="n"/>
       <c r="Z1" s="3" t="n"/>
     </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="3" t="n"/>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="3" t="n"/>
-      <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="n"/>
-      <c r="M2" s="3" t="n"/>
-      <c r="N2" s="3" t="n"/>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
       <c r="O2" s="3" t="n"/>
       <c r="P2" s="3" t="n"/>
       <c r="Q2" s="3" t="n"/>
@@ -8861,35 +8964,15 @@
       <c r="Y2" s="3" t="n"/>
       <c r="Z2" s="3" t="n"/>
     </row>
-    <row r="3" ht="27" customHeight="1">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>Variante recomendada
-Grupo 1</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="n"/>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>Lucro liquido
-R$ 286.570,00</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="n"/>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>Margem GMV
-7,00%</t>
-        </is>
-      </c>
-      <c r="F3" s="9" t="n"/>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>ROI cashback
-175,00%</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="n"/>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="3" t="n"/>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="3" t="n"/>
+      <c r="F3" s="3" t="n"/>
+      <c r="G3" s="3" t="n"/>
+      <c r="H3" s="3" t="n"/>
       <c r="I3" s="3" t="n"/>
       <c r="J3" s="3" t="n"/>
       <c r="K3" s="3" t="n"/>
@@ -8926,13 +9009,33 @@
       <c r="Z3" s="3" t="n"/>
     </row>
     <row r="4" ht="27" customHeight="1">
-      <c r="A4" s="7" t="n"/>
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Variante recomendada
+Grupo 1</t>
+        </is>
+      </c>
       <c r="B4" s="7" t="n"/>
-      <c r="C4" s="7" t="n"/>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Lucro liquido
+R$ 286.570,00</t>
+        </is>
+      </c>
       <c r="D4" s="7" t="n"/>
-      <c r="E4" s="9" t="n"/>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Margem GMV
+7,00%</t>
+        </is>
+      </c>
       <c r="F4" s="9" t="n"/>
-      <c r="G4" s="5" t="n"/>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>ROI cashback
+175,00%</t>
+        </is>
+      </c>
       <c r="H4" s="5" t="n"/>
       <c r="I4" s="3" t="n"/>
       <c r="J4" s="3" t="n"/>
@@ -9001,15 +9104,15 @@
       <c r="Y5" s="3" t="n"/>
       <c r="Z5" s="3" t="n"/>
     </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="3" t="n"/>
-      <c r="B6" s="3" t="n"/>
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
-      <c r="F6" s="3" t="n"/>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
+    <row r="6" ht="27" customHeight="1">
+      <c r="A6" s="7" t="n"/>
+      <c r="B6" s="7" t="n"/>
+      <c r="C6" s="7" t="n"/>
+      <c r="D6" s="7" t="n"/>
+      <c r="E6" s="9" t="n"/>
+      <c r="F6" s="9" t="n"/>
+      <c r="G6" s="5" t="n"/>
+      <c r="H6" s="5" t="n"/>
       <c r="I6" s="3" t="n"/>
       <c r="J6" s="3" t="n"/>
       <c r="K6" s="3" t="n"/>
@@ -9040,22 +9143,14 @@
       <c r="Z6" s="3" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="16" t="inlineStr">
-        <is>
-          <t>Decisao</t>
-        </is>
-      </c>
-      <c r="B7" s="17" t="inlineStr">
-        <is>
-          <t>Escalar Grupo 1 para 100% do trafego, mantendo monitoramento de margem e cashback pago nos primeiros dias.</t>
-        </is>
-      </c>
-      <c r="C7" s="18" t="n"/>
-      <c r="D7" s="18" t="n"/>
-      <c r="E7" s="18" t="n"/>
-      <c r="F7" s="18" t="n"/>
-      <c r="G7" s="18" t="n"/>
-      <c r="H7" s="18" t="n"/>
+      <c r="A7" s="3" t="n"/>
+      <c r="B7" s="3" t="n"/>
+      <c r="C7" s="3" t="n"/>
+      <c r="D7" s="3" t="n"/>
+      <c r="E7" s="3" t="n"/>
+      <c r="F7" s="3" t="n"/>
+      <c r="G7" s="3" t="n"/>
+      <c r="H7" s="3" t="n"/>
       <c r="I7" s="3" t="n"/>
       <c r="J7" s="3" t="n"/>
       <c r="K7" s="3" t="n"/>
@@ -9086,8 +9181,16 @@
       <c r="Z7" s="3" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="18" t="n"/>
-      <c r="B8" s="18" t="n"/>
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>Decisao</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>Escalar Grupo 1 para 100% do trafego, mantendo monitoramento de margem e cashback pago nos primeiros dias.</t>
+        </is>
+      </c>
       <c r="C8" s="18" t="n"/>
       <c r="D8" s="18" t="n"/>
       <c r="E8" s="18" t="n"/>
@@ -9124,14 +9227,14 @@
       <c r="Z8" s="3" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="3" t="n"/>
-      <c r="B9" s="3" t="n"/>
-      <c r="C9" s="3" t="n"/>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
-      <c r="F9" s="3" t="n"/>
-      <c r="G9" s="3" t="n"/>
-      <c r="H9" s="3" t="n"/>
+      <c r="A9" s="18" t="n"/>
+      <c r="B9" s="18" t="n"/>
+      <c r="C9" s="18" t="n"/>
+      <c r="D9" s="18" t="n"/>
+      <c r="E9" s="18" t="n"/>
+      <c r="F9" s="18" t="n"/>
+      <c r="G9" s="18" t="n"/>
+      <c r="H9" s="18" t="n"/>
       <c r="I9" s="3" t="n"/>
       <c r="J9" s="3" t="n"/>
       <c r="K9" s="3" t="n"/>
@@ -9200,46 +9303,14 @@
       <c r="Z10" s="3" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>Grupo</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>Compradores</t>
-        </is>
-      </c>
-      <c r="C11" s="10" t="inlineStr">
-        <is>
-          <t>GMV</t>
-        </is>
-      </c>
-      <c r="D11" s="10" t="inlineStr">
-        <is>
-          <t>Cashback</t>
-        </is>
-      </c>
-      <c r="E11" s="10" t="inlineStr">
-        <is>
-          <t>Lucro</t>
-        </is>
-      </c>
-      <c r="F11" s="10" t="inlineStr">
-        <is>
-          <t>Margem</t>
-        </is>
-      </c>
-      <c r="G11" s="10" t="inlineStr">
-        <is>
-          <t>ROI</t>
-        </is>
-      </c>
-      <c r="H11" s="10" t="inlineStr">
-        <is>
-          <t>Ticket medio</t>
-        </is>
-      </c>
+      <c r="A11" s="3" t="n"/>
+      <c r="B11" s="3" t="n"/>
+      <c r="C11" s="3" t="n"/>
+      <c r="D11" s="3" t="n"/>
+      <c r="E11" s="3" t="n"/>
+      <c r="F11" s="3" t="n"/>
+      <c r="G11" s="3" t="n"/>
+      <c r="H11" s="3" t="n"/>
       <c r="I11" s="3" t="n"/>
       <c r="J11" s="3" t="n"/>
       <c r="K11" s="3" t="n"/>
@@ -9270,31 +9341,45 @@
       <c r="Z11" s="3" t="n"/>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>Grupo 1</t>
-        </is>
-      </c>
-      <c r="B12" s="19" t="n">
-        <v>7990</v>
-      </c>
-      <c r="C12" s="20" t="n">
-        <v>4093818</v>
-      </c>
-      <c r="D12" s="20" t="n">
-        <v>163751</v>
-      </c>
-      <c r="E12" s="20" t="n">
-        <v>286570</v>
-      </c>
-      <c r="F12" s="21" t="n">
-        <v>0.07000066930185954</v>
-      </c>
-      <c r="G12" s="21" t="n">
-        <v>1.750035114289378</v>
-      </c>
-      <c r="H12" s="20" t="n">
-        <v>512.3677096370463</v>
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Grupo</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Compradores</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>GMV</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>Cashback</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>Lucro</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>Margem</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>ROI</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>Ticket medio</t>
+        </is>
       </c>
       <c r="I12" s="3" t="n"/>
       <c r="J12" s="3" t="n"/>
@@ -9326,31 +9411,31 @@
       <c r="Z12" s="3" t="n"/>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="11" t="inlineStr">
-        <is>
-          <t>Grupo 2</t>
-        </is>
-      </c>
-      <c r="B13" s="11" t="n">
-        <v>5452</v>
-      </c>
-      <c r="C13" s="12" t="n">
-        <v>2863019</v>
-      </c>
-      <c r="D13" s="12" t="n">
-        <v>171778</v>
-      </c>
-      <c r="E13" s="12" t="n">
-        <v>143157</v>
-      </c>
-      <c r="F13" s="13" t="n">
-        <v>0.05000211315398186</v>
-      </c>
-      <c r="G13" s="13" t="n">
-        <v>0.8333837860494359</v>
-      </c>
-      <c r="H13" s="12" t="n">
-        <v>525.1318782098313</v>
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>Grupo 1</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="n">
+        <v>7990</v>
+      </c>
+      <c r="C13" s="20" t="n">
+        <v>4093818</v>
+      </c>
+      <c r="D13" s="20" t="n">
+        <v>163751</v>
+      </c>
+      <c r="E13" s="20" t="n">
+        <v>286570</v>
+      </c>
+      <c r="F13" s="21" t="n">
+        <v>0.07000066930185954</v>
+      </c>
+      <c r="G13" s="21" t="n">
+        <v>1.750035114289378</v>
+      </c>
+      <c r="H13" s="20" t="n">
+        <v>512.3677096370463</v>
       </c>
       <c r="I13" s="3" t="n"/>
       <c r="J13" s="3" t="n"/>
@@ -9384,29 +9469,29 @@
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>Grupo 3</t>
+          <t>Grupo 2</t>
         </is>
       </c>
       <c r="B14" s="11" t="n">
-        <v>5029</v>
+        <v>5452</v>
       </c>
       <c r="C14" s="12" t="n">
-        <v>2629963</v>
+        <v>2863019</v>
       </c>
       <c r="D14" s="12" t="n">
-        <v>236697</v>
+        <v>171778</v>
       </c>
       <c r="E14" s="12" t="n">
-        <v>52593</v>
+        <v>143157</v>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.01999761973837655</v>
+        <v>0.05000211315398186</v>
       </c>
       <c r="G14" s="13" t="n">
-        <v>0.2221954650882774</v>
+        <v>0.8333837860494359</v>
       </c>
       <c r="H14" s="12" t="n">
-        <v>522.9594352754027</v>
+        <v>525.1318782098313</v>
       </c>
       <c r="I14" s="3" t="n"/>
       <c r="J14" s="3" t="n"/>
@@ -9438,14 +9523,32 @@
       <c r="Z14" s="3" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="3" t="n"/>
-      <c r="B15" s="3" t="n"/>
-      <c r="C15" s="3" t="n"/>
-      <c r="D15" s="3" t="n"/>
-      <c r="E15" s="3" t="n"/>
-      <c r="F15" s="3" t="n"/>
-      <c r="G15" s="3" t="n"/>
-      <c r="H15" s="3" t="n"/>
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>Grupo 3</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="n">
+        <v>5029</v>
+      </c>
+      <c r="C15" s="12" t="n">
+        <v>2629963</v>
+      </c>
+      <c r="D15" s="12" t="n">
+        <v>236697</v>
+      </c>
+      <c r="E15" s="12" t="n">
+        <v>52593</v>
+      </c>
+      <c r="F15" s="13" t="n">
+        <v>0.01999761973837655</v>
+      </c>
+      <c r="G15" s="13" t="n">
+        <v>0.2221954650882774</v>
+      </c>
+      <c r="H15" s="12" t="n">
+        <v>522.9594352754027</v>
+      </c>
       <c r="I15" s="3" t="n"/>
       <c r="J15" s="3" t="n"/>
       <c r="K15" s="3" t="n"/>
@@ -12907,12 +13010,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A1:N1"/>
-    <mergeCell ref="A3:B5"/>
-    <mergeCell ref="G3:H5"/>
-    <mergeCell ref="E3:F5"/>
-    <mergeCell ref="B7:H8"/>
-    <mergeCell ref="C3:D5"/>
+    <mergeCell ref="A1:N2"/>
+    <mergeCell ref="E4:F6"/>
+    <mergeCell ref="B8:H9"/>
+    <mergeCell ref="C4:D6"/>
+    <mergeCell ref="A4:B6"/>
+    <mergeCell ref="G4:H6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -12956,10 +13059,11 @@
     <col width="12" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Teste cashback - Parceiro C</t>
+          <t xml:space="preserve">     Teste cashback - Parceiro C
+     2011-07-01 a 2011-08-14 | decisao automatizada</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -12992,21 +13096,21 @@
       <c r="Y1" s="3" t="n"/>
       <c r="Z1" s="3" t="n"/>
     </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="3" t="n"/>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="3" t="n"/>
-      <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="n"/>
-      <c r="M2" s="3" t="n"/>
-      <c r="N2" s="3" t="n"/>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
       <c r="O2" s="3" t="n"/>
       <c r="P2" s="3" t="n"/>
       <c r="Q2" s="3" t="n"/>
@@ -13020,35 +13124,15 @@
       <c r="Y2" s="3" t="n"/>
       <c r="Z2" s="3" t="n"/>
     </row>
-    <row r="3" ht="27" customHeight="1">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>Variante recomendada
-Grupo 1</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="n"/>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>Lucro liquido
-R$ 34.769,00</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="n"/>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>Margem GMV
-2,00%</t>
-        </is>
-      </c>
-      <c r="F3" s="9" t="n"/>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>ROI cashback
-40,00%</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="n"/>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="3" t="n"/>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="3" t="n"/>
+      <c r="F3" s="3" t="n"/>
+      <c r="G3" s="3" t="n"/>
+      <c r="H3" s="3" t="n"/>
       <c r="I3" s="3" t="n"/>
       <c r="J3" s="3" t="n"/>
       <c r="K3" s="3" t="n"/>
@@ -13081,13 +13165,33 @@
       <c r="Z3" s="3" t="n"/>
     </row>
     <row r="4" ht="27" customHeight="1">
-      <c r="A4" s="7" t="n"/>
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Variante recomendada
+Grupo 1</t>
+        </is>
+      </c>
       <c r="B4" s="7" t="n"/>
-      <c r="C4" s="7" t="n"/>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Lucro liquido
+R$ 34.769,00</t>
+        </is>
+      </c>
       <c r="D4" s="7" t="n"/>
-      <c r="E4" s="9" t="n"/>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Margem GMV
+2,00%</t>
+        </is>
+      </c>
       <c r="F4" s="9" t="n"/>
-      <c r="G4" s="5" t="n"/>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>ROI cashback
+40,00%</t>
+        </is>
+      </c>
       <c r="H4" s="5" t="n"/>
       <c r="I4" s="3" t="n"/>
       <c r="J4" s="3" t="n"/>
@@ -13152,15 +13256,15 @@
       <c r="Y5" s="3" t="n"/>
       <c r="Z5" s="3" t="n"/>
     </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="3" t="n"/>
-      <c r="B6" s="3" t="n"/>
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
-      <c r="F6" s="3" t="n"/>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
+    <row r="6" ht="27" customHeight="1">
+      <c r="A6" s="7" t="n"/>
+      <c r="B6" s="7" t="n"/>
+      <c r="C6" s="7" t="n"/>
+      <c r="D6" s="7" t="n"/>
+      <c r="E6" s="9" t="n"/>
+      <c r="F6" s="9" t="n"/>
+      <c r="G6" s="5" t="n"/>
+      <c r="H6" s="5" t="n"/>
       <c r="I6" s="3" t="n"/>
       <c r="J6" s="3" t="n"/>
       <c r="K6" s="3" t="n"/>
@@ -13189,22 +13293,14 @@
       <c r="Z6" s="3" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="16" t="inlineStr">
-        <is>
-          <t>Decisao</t>
-        </is>
-      </c>
-      <c r="B7" s="17" t="inlineStr">
-        <is>
-          <t>Escalar Grupo 1 para 100% do trafego, mantendo monitoramento de margem e cashback pago nos primeiros dias.</t>
-        </is>
-      </c>
-      <c r="C7" s="18" t="n"/>
-      <c r="D7" s="18" t="n"/>
-      <c r="E7" s="18" t="n"/>
-      <c r="F7" s="18" t="n"/>
-      <c r="G7" s="18" t="n"/>
-      <c r="H7" s="18" t="n"/>
+      <c r="A7" s="3" t="n"/>
+      <c r="B7" s="3" t="n"/>
+      <c r="C7" s="3" t="n"/>
+      <c r="D7" s="3" t="n"/>
+      <c r="E7" s="3" t="n"/>
+      <c r="F7" s="3" t="n"/>
+      <c r="G7" s="3" t="n"/>
+      <c r="H7" s="3" t="n"/>
       <c r="I7" s="3" t="n"/>
       <c r="J7" s="3" t="n"/>
       <c r="K7" s="3" t="n"/>
@@ -13233,8 +13329,16 @@
       <c r="Z7" s="3" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="18" t="n"/>
-      <c r="B8" s="18" t="n"/>
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>Decisao</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>Escalar Grupo 1 para 100% do trafego, mantendo monitoramento de margem e cashback pago nos primeiros dias.</t>
+        </is>
+      </c>
       <c r="C8" s="18" t="n"/>
       <c r="D8" s="18" t="n"/>
       <c r="E8" s="18" t="n"/>
@@ -13269,14 +13373,14 @@
       <c r="Z8" s="3" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="3" t="n"/>
-      <c r="B9" s="3" t="n"/>
-      <c r="C9" s="3" t="n"/>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
-      <c r="F9" s="3" t="n"/>
-      <c r="G9" s="3" t="n"/>
-      <c r="H9" s="3" t="n"/>
+      <c r="A9" s="18" t="n"/>
+      <c r="B9" s="18" t="n"/>
+      <c r="C9" s="18" t="n"/>
+      <c r="D9" s="18" t="n"/>
+      <c r="E9" s="18" t="n"/>
+      <c r="F9" s="18" t="n"/>
+      <c r="G9" s="18" t="n"/>
+      <c r="H9" s="18" t="n"/>
       <c r="I9" s="3" t="n"/>
       <c r="J9" s="3" t="n"/>
       <c r="K9" s="3" t="n"/>
@@ -13341,46 +13445,14 @@
       <c r="Z10" s="3" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>Grupo</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>Compradores</t>
-        </is>
-      </c>
-      <c r="C11" s="10" t="inlineStr">
-        <is>
-          <t>GMV</t>
-        </is>
-      </c>
-      <c r="D11" s="10" t="inlineStr">
-        <is>
-          <t>Cashback</t>
-        </is>
-      </c>
-      <c r="E11" s="10" t="inlineStr">
-        <is>
-          <t>Lucro</t>
-        </is>
-      </c>
-      <c r="F11" s="10" t="inlineStr">
-        <is>
-          <t>Margem</t>
-        </is>
-      </c>
-      <c r="G11" s="10" t="inlineStr">
-        <is>
-          <t>ROI</t>
-        </is>
-      </c>
-      <c r="H11" s="10" t="inlineStr">
-        <is>
-          <t>Ticket medio</t>
-        </is>
-      </c>
+      <c r="A11" s="3" t="n"/>
+      <c r="B11" s="3" t="n"/>
+      <c r="C11" s="3" t="n"/>
+      <c r="D11" s="3" t="n"/>
+      <c r="E11" s="3" t="n"/>
+      <c r="F11" s="3" t="n"/>
+      <c r="G11" s="3" t="n"/>
+      <c r="H11" s="3" t="n"/>
       <c r="I11" s="3" t="n"/>
       <c r="J11" s="3" t="n"/>
       <c r="K11" s="3" t="n"/>
@@ -13409,31 +13481,45 @@
       <c r="Z11" s="3" t="n"/>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>Grupo 1</t>
-        </is>
-      </c>
-      <c r="B12" s="19" t="n">
-        <v>4549</v>
-      </c>
-      <c r="C12" s="20" t="n">
-        <v>1738460</v>
-      </c>
-      <c r="D12" s="20" t="n">
-        <v>86924</v>
-      </c>
-      <c r="E12" s="20" t="n">
-        <v>34769</v>
-      </c>
-      <c r="F12" s="21" t="n">
-        <v>0.0199998849556504</v>
-      </c>
-      <c r="G12" s="21" t="n">
-        <v>0.3999930974184345</v>
-      </c>
-      <c r="H12" s="20" t="n">
-        <v>382.1631127720378</v>
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Grupo</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Compradores</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>GMV</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>Cashback</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>Lucro</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>Margem</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>ROI</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>Ticket medio</t>
+        </is>
       </c>
       <c r="I12" s="3" t="n"/>
       <c r="J12" s="3" t="n"/>
@@ -13463,31 +13549,31 @@
       <c r="Z12" s="3" t="n"/>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="11" t="inlineStr">
-        <is>
-          <t>Grupo 2</t>
-        </is>
-      </c>
-      <c r="B13" s="11" t="n">
-        <v>4522</v>
-      </c>
-      <c r="C13" s="12" t="n">
-        <v>1685235</v>
-      </c>
-      <c r="D13" s="12" t="n">
-        <v>117967</v>
-      </c>
-      <c r="E13" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="12" t="n">
-        <v>372.6747014595312</v>
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>Grupo 1</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="n">
+        <v>4549</v>
+      </c>
+      <c r="C13" s="20" t="n">
+        <v>1738460</v>
+      </c>
+      <c r="D13" s="20" t="n">
+        <v>86924</v>
+      </c>
+      <c r="E13" s="20" t="n">
+        <v>34769</v>
+      </c>
+      <c r="F13" s="21" t="n">
+        <v>0.0199998849556504</v>
+      </c>
+      <c r="G13" s="21" t="n">
+        <v>0.3999930974184345</v>
+      </c>
+      <c r="H13" s="20" t="n">
+        <v>382.1631127720378</v>
       </c>
       <c r="I13" s="3" t="n"/>
       <c r="J13" s="3" t="n"/>
@@ -13517,14 +13603,32 @@
       <c r="Z13" s="3" t="n"/>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="3" t="n"/>
-      <c r="B14" s="3" t="n"/>
-      <c r="C14" s="3" t="n"/>
-      <c r="D14" s="3" t="n"/>
-      <c r="E14" s="3" t="n"/>
-      <c r="F14" s="3" t="n"/>
-      <c r="G14" s="3" t="n"/>
-      <c r="H14" s="3" t="n"/>
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>Grupo 2</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="n">
+        <v>4522</v>
+      </c>
+      <c r="C14" s="12" t="n">
+        <v>1685235</v>
+      </c>
+      <c r="D14" s="12" t="n">
+        <v>117967</v>
+      </c>
+      <c r="E14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="12" t="n">
+        <v>372.6747014595312</v>
+      </c>
       <c r="I14" s="3" t="n"/>
       <c r="J14" s="3" t="n"/>
       <c r="K14" s="3" t="n"/>
@@ -16794,12 +16898,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A1:N1"/>
-    <mergeCell ref="A3:B5"/>
-    <mergeCell ref="G3:H5"/>
-    <mergeCell ref="E3:F5"/>
-    <mergeCell ref="B7:H8"/>
-    <mergeCell ref="C3:D5"/>
+    <mergeCell ref="A1:N2"/>
+    <mergeCell ref="E4:F6"/>
+    <mergeCell ref="B8:H9"/>
+    <mergeCell ref="C4:D6"/>
+    <mergeCell ref="A4:B6"/>
+    <mergeCell ref="G4:H6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>